<commit_message>
update and push readme
</commit_message>
<xml_diff>
--- a/outbreaks/data/dx_readiness_comp_data_20250212.xlsx
+++ b/outbreaks/data/dx_readiness_comp_data_20250212.xlsx
@@ -1097,7 +1097,7 @@
         <v>28</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1183,7 +1183,7 @@
         <v>111</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">

</xml_diff>